<commit_message>
fix: return method-not-allowed envelopes and refresh round 2
</commit_message>
<xml_diff>
--- a/outputs/pbl6-round2/Test_Report_API_Postman_Round2.xlsx
+++ b/outputs/pbl6-round2/Test_Report_API_Postman_Round2.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Read39d528c014fe5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" r:id="R0c66f25a7f3a45ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Statistics" sheetId="3" r:id="Rc82aa1b74d644d97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auth_Service" sheetId="4" r:id="R1d3d4a0f86e645b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trip_Service" sheetId="5" r:id="R3edb62e4574f4ccb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Booking_Service" sheetId="6" r:id="R716822149f6e4508"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payment_Service" sheetId="7" r:id="R34cf01215ac143c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notification_Service" sheetId="8" r:id="Re64f6718c1a4411f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report_Service" sheetId="9" r:id="R8c0475b5e4054dc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Round2_Evidence" sheetId="10" r:id="R10efc6eea56948e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rbaa22682868844bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" r:id="R4f38798d2ba049bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Statistics" sheetId="3" r:id="R7ced2bc7ba834230"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auth_Service" sheetId="4" r:id="R4b0d25d509b044b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trip_Service" sheetId="5" r:id="Ra102f4d1d7c849f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Booking_Service" sheetId="6" r:id="R4fbeafc7420c469c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payment_Service" sheetId="7" r:id="R1ba5b6616aa54618"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notification_Service" sheetId="8" r:id="R3a42a2e8d47047f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report_Service" sheetId="9" r:id="Ra46cebe1d86742d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Round2_Evidence" sheetId="10" r:id="Ra273fa1176984bc0"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="ACTION">#REF!</x:definedName>
@@ -4793,7 +4793,7 @@
     <x:mergeCell ref="B4:D4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9aa051fe58cb44ef"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R931ec0d482cc47d0"/>
 </x:worksheet>
 </file>
 
@@ -4878,7 +4878,7 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="I3" t="str">
-        <x:v>38 clean / 34 with failures</x:v>
+        <x:v>39 clean / 33 with failures</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -4889,14 +4889,14 @@
         <x:v>421</x:v>
       </x:c>
       <x:c r="C4" t="n">
-        <x:v>358</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="D4" t="n">
-        <x:v>63</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="E4" s="164" t="n">
         <x:f>C4/B4</x:f>
-        <x:v>0.850356294536817</x:v>
+        <x:v>0.8551068883610451</x:v>
       </x:c>
       <x:c r="G4" t="str">
         <x:v>Target</x:v>
@@ -4915,21 +4915,21 @@
       <x:c r="B5"/>
       <x:c r="C5" t="n">
         <x:f>C4-C3</x:f>
-        <x:v>28</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D5" t="n">
         <x:f>D4-D3</x:f>
-        <x:v>-26</x:v>
+        <x:v>-28</x:v>
       </x:c>
       <x:c r="E5" s="164" t="n">
         <x:f>E4-E3</x:f>
-        <x:v>0.06276679573013444</x:v>
+        <x:v>0.06751738955436248</x:v>
       </x:c>
       <x:c r="G5" t="str">
         <x:v>Completed UTC</x:v>
       </x:c>
       <x:c r="H5" s="165" t="d">
-        <x:v>2026-10-30T04:02:18.216Z</x:v>
+        <x:v>2026-10-30T04:18:36.356Z</x:v>
       </x:c>
       <x:c r="I5" t="str">
         <x:v>Evidence retained</x:v>
@@ -4997,7 +4997,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G11" s="173" t="n">
-        <x:v>2.551</x:v>
+        <x:v>2.995</x:v>
       </x:c>
       <x:c r="H11" s="175" t="str">
         <x:v>logs/PBL6_PAY03_Readback.postman_collection.log</x:v>
@@ -5026,7 +5026,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G12" s="173" t="n">
-        <x:v>3.361</x:v>
+        <x:v>2.433</x:v>
       </x:c>
       <x:c r="H12" s="175" t="str">
         <x:v>logs/PBL6_R3_AdminRoles.postman_collection.log</x:v>
@@ -5055,7 +5055,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G13" s="173" t="n">
-        <x:v>2.519</x:v>
+        <x:v>2.46</x:v>
       </x:c>
       <x:c r="H13" s="175" t="str">
         <x:v>logs/PBL6_R3_AdminSettlement.postman_collection.log</x:v>
@@ -5084,7 +5084,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G14" s="173" t="n">
-        <x:v>4.176</x:v>
+        <x:v>3.814</x:v>
       </x:c>
       <x:c r="H14" s="175" t="str">
         <x:v>logs/PBL6_R3_Auth_Common_Security.postman_collection.log</x:v>
@@ -5113,7 +5113,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G15" s="173" t="n">
-        <x:v>2.44</x:v>
+        <x:v>2.534</x:v>
       </x:c>
       <x:c r="H15" s="175" t="str">
         <x:v>logs/PBL6_R3_AuthExpiry.postman_collection.log</x:v>
@@ -5142,7 +5142,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G16" s="173" t="n">
-        <x:v>2.441</x:v>
+        <x:v>2.206</x:v>
       </x:c>
       <x:c r="H16" s="175" t="str">
         <x:v>logs/PBL6_R3_CreateSecondCustomer.postman_collection.log</x:v>
@@ -5171,7 +5171,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G17" s="173" t="n">
-        <x:v>2.397</x:v>
+        <x:v>2.485</x:v>
       </x:c>
       <x:c r="H17" s="175" t="str">
         <x:v>logs/PBL6_R3_BOOK03_BOOK04_ExistingTrip.postman_collection.log</x:v>
@@ -5200,7 +5200,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G18" s="173" t="n">
-        <x:v>3.262</x:v>
+        <x:v>3.853</x:v>
       </x:c>
       <x:c r="H18" s="175" t="str">
         <x:v>logs/PBL6_R3_BOOK03_BOOK04_Multiseat.postman_collection.log</x:v>
@@ -5229,7 +5229,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G19" s="173" t="n">
-        <x:v>1.973</x:v>
+        <x:v>2.02</x:v>
       </x:c>
       <x:c r="H19" s="175" t="str">
         <x:v>logs/PBL6_R3_BOOK05_ConcurrentHold.postman_collection.log</x:v>
@@ -5258,7 +5258,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G20" s="173" t="n">
-        <x:v>2.53</x:v>
+        <x:v>2.111</x:v>
       </x:c>
       <x:c r="H20" s="175" t="str">
         <x:v>logs/PBL6_R3_BOOK12_BOOK13_PayLaterIdempotency.postman_collection.log</x:v>
@@ -5316,7 +5316,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G22" s="173" t="n">
-        <x:v>2.057</x:v>
+        <x:v>1.965</x:v>
       </x:c>
       <x:c r="H22" s="175" t="str">
         <x:v>logs/PBL6_R3_BOOK18_PayLater.postman_collection.log</x:v>
@@ -5345,7 +5345,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G23" s="173" t="n">
-        <x:v>2.237</x:v>
+        <x:v>2.002</x:v>
       </x:c>
       <x:c r="H23" s="175" t="str">
         <x:v>logs/PBL6_R3_BOOK20_InvalidChannel.postman_collection.log</x:v>
@@ -5374,7 +5374,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G24" s="173" t="n">
-        <x:v>2.358</x:v>
+        <x:v>2.257</x:v>
       </x:c>
       <x:c r="H24" s="175" t="str">
         <x:v>logs/PBL6_R3_Booking.postman_collection.log</x:v>
@@ -5403,7 +5403,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G25" s="173" t="n">
-        <x:v>2.226</x:v>
+        <x:v>2.027</x:v>
       </x:c>
       <x:c r="H25" s="175" t="str">
         <x:v>logs/PBL6_R3_BookingCorrectTotal.postman_collection.log</x:v>
@@ -5432,7 +5432,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G26" s="173" t="n">
-        <x:v>2.031</x:v>
+        <x:v>2.263</x:v>
       </x:c>
       <x:c r="H26" s="175" t="str">
         <x:v>logs/PBL6_R3_BookingExpiry.postman_collection.log</x:v>
@@ -5461,7 +5461,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G27" s="173" t="n">
-        <x:v>4.272</x:v>
+        <x:v>3.462</x:v>
       </x:c>
       <x:c r="H27" s="175" t="str">
         <x:v>logs/PBL6_R3_BookingFresh.postman_collection.log</x:v>
@@ -5490,7 +5490,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G28" s="173" t="n">
-        <x:v>2.056</x:v>
+        <x:v>2.235</x:v>
       </x:c>
       <x:c r="H28" s="175" t="str">
         <x:v>logs/PBL6_R3_BookingInvalidChannel.postman_collection.log</x:v>
@@ -5519,7 +5519,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G29" s="173" t="n">
-        <x:v>2.24</x:v>
+        <x:v>2.117</x:v>
       </x:c>
       <x:c r="H29" s="175" t="str">
         <x:v>logs/PBL6_R3_BookingState.postman_collection.log</x:v>
@@ -5548,7 +5548,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G30" s="173" t="n">
-        <x:v>2.196</x:v>
+        <x:v>2.361</x:v>
       </x:c>
       <x:c r="H30" s="175" t="str">
         <x:v>logs/PBL6_R3_BookingValidation.postman_collection.log</x:v>
@@ -5577,7 +5577,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G31" s="173" t="n">
-        <x:v>2.11</x:v>
+        <x:v>1.978</x:v>
       </x:c>
       <x:c r="H31" s="175" t="str">
         <x:v>logs/PBL6_R3_CAN01_Preview.postman_collection.log</x:v>
@@ -5606,7 +5606,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G32" s="173" t="n">
-        <x:v>2.107</x:v>
+        <x:v>2.352</x:v>
       </x:c>
       <x:c r="H32" s="175" t="str">
         <x:v>logs/PBL6_R3_CAN02_PrepaidConfirmCancel.postman_collection.log</x:v>
@@ -5635,7 +5635,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G33" s="173" t="n">
-        <x:v>4.103</x:v>
+        <x:v>5.819</x:v>
       </x:c>
       <x:c r="H33" s="175" t="str">
         <x:v>logs/PBL6_R3_CAN02_PrepaidRefundFlow.postman_collection.log</x:v>
@@ -5664,7 +5664,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G34" s="173" t="n">
-        <x:v>2.096</x:v>
+        <x:v>2.074</x:v>
       </x:c>
       <x:c r="H34" s="175" t="str">
         <x:v>logs/PBL6_R3_CAN02_RefundReadback.postman_collection.log</x:v>
@@ -5693,7 +5693,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G35" s="173" t="n">
-        <x:v>2.99</x:v>
+        <x:v>2.175</x:v>
       </x:c>
       <x:c r="H35" s="175" t="str">
         <x:v>logs/PBL6_R3_CAN03_PayLaterCancellation.postman_collection.log</x:v>
@@ -5722,7 +5722,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G36" s="173" t="n">
-        <x:v>2.046</x:v>
+        <x:v>2.025</x:v>
       </x:c>
       <x:c r="H36" s="175" t="str">
         <x:v>logs/PBL6_R3_CAN04_CancelReplay.postman_collection.log</x:v>
@@ -5751,7 +5751,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G37" s="173" t="n">
-        <x:v>2.283</x:v>
+        <x:v>2.084</x:v>
       </x:c>
       <x:c r="H37" s="175" t="str">
         <x:v>logs/PBL6_R3_CAN05_CheckedIn.postman_collection.log</x:v>
@@ -5780,7 +5780,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G38" s="173" t="n">
-        <x:v>2.191</x:v>
+        <x:v>1.995</x:v>
       </x:c>
       <x:c r="H38" s="175" t="str">
         <x:v>logs/PBL6_R3_CAN06_RepeatCancelled.postman_collection.log</x:v>
@@ -5809,7 +5809,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G39" s="173" t="n">
-        <x:v>2.339</x:v>
+        <x:v>1.942</x:v>
       </x:c>
       <x:c r="H39" s="175" t="str">
         <x:v>logs/PBL6_R3_CAN09_ForeignPreview.postman_collection.log</x:v>
@@ -5838,7 +5838,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G40" s="173" t="n">
-        <x:v>2.264</x:v>
+        <x:v>2.122</x:v>
       </x:c>
       <x:c r="H40" s="175" t="str">
         <x:v>logs/PBL6_R3_CancelledTripHold.postman_collection.log</x:v>
@@ -5867,7 +5867,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G41" s="173" t="n">
-        <x:v>2.416</x:v>
+        <x:v>2.52</x:v>
       </x:c>
       <x:c r="H41" s="175" t="str">
         <x:v>logs/PBL6_R3_CommonFormats.postman_collection.log</x:v>
@@ -5896,7 +5896,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G42" s="173" t="n">
-        <x:v>2.742</x:v>
+        <x:v>2.4</x:v>
       </x:c>
       <x:c r="H42" s="175" t="str">
         <x:v>logs/PBL6_R3_CrossTenant.postman_collection.log</x:v>
@@ -5925,7 +5925,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G43" s="173" t="n">
-        <x:v>2.482</x:v>
+        <x:v>2.522</x:v>
       </x:c>
       <x:c r="H43" s="175" t="str">
         <x:v>logs/PBL6_R3_Drivers.postman_collection.log</x:v>
@@ -5954,7 +5954,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G44" s="173" t="n">
-        <x:v>2.348</x:v>
+        <x:v>2.77</x:v>
       </x:c>
       <x:c r="H44" s="175" t="str">
         <x:v>logs/PBL6_R3_DriverScheduleConflict.postman_collection.log</x:v>
@@ -5983,7 +5983,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G45" s="173" t="n">
-        <x:v>2.251</x:v>
+        <x:v>2.268</x:v>
       </x:c>
       <x:c r="H45" s="175" t="str">
         <x:v>logs/PBL6_R3_ExpiredHoldBooking.postman_collection.log</x:v>
@@ -6012,7 +6012,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G46" s="173" t="n">
-        <x:v>2.044</x:v>
+        <x:v>2.073</x:v>
       </x:c>
       <x:c r="H46" s="175" t="str">
         <x:v>logs/PBL6_R3_ExpiredToken.postman_collection.log</x:v>
@@ -6041,7 +6041,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G47" s="173" t="n">
-        <x:v>2.493</x:v>
+        <x:v>2.141</x:v>
       </x:c>
       <x:c r="H47" s="175" t="str">
         <x:v>logs/PBL6_R3_FinalAdmin.postman_collection.log</x:v>
@@ -6070,7 +6070,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G48" s="173" t="n">
-        <x:v>1.89</x:v>
+        <x:v>2.117</x:v>
       </x:c>
       <x:c r="H48" s="175" t="str">
         <x:v>logs/PBL6_R3_HoldExpiry.postman_collection.log</x:v>
@@ -6099,7 +6099,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G49" s="173" t="n">
-        <x:v>2.163</x:v>
+        <x:v>2.188</x:v>
       </x:c>
       <x:c r="H49" s="175" t="str">
         <x:v>logs/PBL6_R3_NotificationSettlement.postman_collection.log</x:v>
@@ -6128,7 +6128,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G50" s="173" t="n">
-        <x:v>2.268</x:v>
+        <x:v>1.913</x:v>
       </x:c>
       <x:c r="H50" s="175" t="str">
         <x:v>logs/PBL6_R3_OrganizationMember.postman_collection.log</x:v>
@@ -6157,7 +6157,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G51" s="173" t="n">
-        <x:v>3.688</x:v>
+        <x:v>3.337</x:v>
       </x:c>
       <x:c r="H51" s="175" t="str">
         <x:v>logs/PBL6_R3_PAY11_NoWebhook.postman_collection.log</x:v>
@@ -6186,7 +6186,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G52" s="173" t="n">
-        <x:v>2.231</x:v>
+        <x:v>2.133</x:v>
       </x:c>
       <x:c r="H52" s="175" t="str">
         <x:v>logs/PBL6_R3_PaymentAmount.postman_collection.log</x:v>
@@ -6215,7 +6215,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G53" s="173" t="n">
-        <x:v>5.431</x:v>
+        <x:v>5.407</x:v>
       </x:c>
       <x:c r="H53" s="175" t="str">
         <x:v>logs/PBL6_R3_PaymentAmountSigned.postman_collection.log</x:v>
@@ -6244,7 +6244,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G54" s="173" t="n">
-        <x:v>2.163</x:v>
+        <x:v>2.447</x:v>
       </x:c>
       <x:c r="H54" s="175" t="str">
         <x:v>logs/PBL6_R3_PaymentComplete.postman_collection.log</x:v>
@@ -6273,7 +6273,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G55" s="173" t="n">
-        <x:v>2.241</x:v>
+        <x:v>2.529</x:v>
       </x:c>
       <x:c r="H55" s="175" t="str">
         <x:v>logs/PBL6_R3_PaymentFailure.postman_collection.log</x:v>
@@ -6302,7 +6302,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G56" s="173" t="n">
-        <x:v>5.207</x:v>
+        <x:v>5.514</x:v>
       </x:c>
       <x:c r="H56" s="175" t="str">
         <x:v>logs/PBL6_R3_PaymentIdempotency.postman_collection.log</x:v>
@@ -6331,7 +6331,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G57" s="173" t="n">
-        <x:v>3.691</x:v>
+        <x:v>2.102</x:v>
       </x:c>
       <x:c r="H57" s="175" t="str">
         <x:v>logs/PBL6_R3_PaymentIntent.postman_collection.log</x:v>
@@ -6360,7 +6360,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G58" s="173" t="n">
-        <x:v>1.943</x:v>
+        <x:v>2.17</x:v>
       </x:c>
       <x:c r="H58" s="175" t="str">
         <x:v>logs/PBL6_R3_PaymentReadback.postman_collection.log</x:v>
@@ -6389,7 +6389,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G59" s="173" t="n">
-        <x:v>2.158</x:v>
+        <x:v>2.75</x:v>
       </x:c>
       <x:c r="H59" s="175" t="str">
         <x:v>logs/PBL6_R3_ProfileEmail.postman_collection.log</x:v>
@@ -6418,7 +6418,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G60" s="173" t="n">
-        <x:v>2.078</x:v>
+        <x:v>1.945</x:v>
       </x:c>
       <x:c r="H60" s="175" t="str">
         <x:v>logs/PBL6_R3_ReadSyntheticTrip.postman_collection.log</x:v>
@@ -6447,7 +6447,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G61" s="173" t="n">
-        <x:v>2.102</x:v>
+        <x:v>1.916</x:v>
       </x:c>
       <x:c r="H61" s="175" t="str">
         <x:v>logs/PBL6_R3_ReadTripSevenSeats.postman_collection.log</x:v>
@@ -6476,7 +6476,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G62" s="173" t="n">
-        <x:v>2.879</x:v>
+        <x:v>2.166</x:v>
       </x:c>
       <x:c r="H62" s="175" t="str">
         <x:v>logs/PBL6_R3_ReportReadback.postman_collection.log</x:v>
@@ -6505,7 +6505,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G63" s="173" t="n">
-        <x:v>1.981</x:v>
+        <x:v>2.138</x:v>
       </x:c>
       <x:c r="H63" s="175" t="str">
         <x:v>logs/PBL6_R3_Resource_Readback.postman_collection.log</x:v>
@@ -6534,7 +6534,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G64" s="173" t="n">
-        <x:v>2.153</x:v>
+        <x:v>2.155</x:v>
       </x:c>
       <x:c r="H64" s="175" t="str">
         <x:v>logs/PBL6_R3_SearchLimit.postman_collection.log</x:v>
@@ -6563,7 +6563,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G65" s="173" t="n">
-        <x:v>2.186</x:v>
+        <x:v>2.173</x:v>
       </x:c>
       <x:c r="H65" s="175" t="str">
         <x:v>logs/PBL6_R3_SearchNotSellable.postman_collection.log</x:v>
@@ -6592,7 +6592,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G66" s="173" t="n">
-        <x:v>2.685</x:v>
+        <x:v>2.127</x:v>
       </x:c>
       <x:c r="H66" s="175" t="str">
         <x:v>logs/PBL6_R3_SeatReadback.postman_collection.log</x:v>
@@ -6621,7 +6621,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G67" s="173" t="n">
-        <x:v>3.062</x:v>
+        <x:v>2.483</x:v>
       </x:c>
       <x:c r="H67" s="175" t="str">
         <x:v>logs/PBL6_R3_SecurityRateInjection.postman_collection.log</x:v>
@@ -6650,7 +6650,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G68" s="173" t="n">
-        <x:v>2.279</x:v>
+        <x:v>2.359</x:v>
       </x:c>
       <x:c r="H68" s="175" t="str">
         <x:v>logs/PBL6_R3_TicketCheckin.postman_collection.log</x:v>
@@ -6679,7 +6679,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G69" s="173" t="n">
-        <x:v>2.134</x:v>
+        <x:v>2.445</x:v>
       </x:c>
       <x:c r="H69" s="175" t="str">
         <x:v>logs/PBL6_R3_TKT08_CancelledTripScan.postman_collection.log</x:v>
@@ -6708,7 +6708,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G70" s="173" t="n">
-        <x:v>2.147</x:v>
+        <x:v>2.028</x:v>
       </x:c>
       <x:c r="H70" s="175" t="str">
         <x:v>logs/PBL6_R3_TKT09_CustomerCheckin.postman_collection.log</x:v>
@@ -6737,7 +6737,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G71" s="173" t="n">
-        <x:v>2.328</x:v>
+        <x:v>2.071</x:v>
       </x:c>
       <x:c r="H71" s="175" t="str">
         <x:v>logs/PBL6_R3_Transport.postman_collection.log</x:v>
@@ -6766,7 +6766,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G72" s="173" t="n">
-        <x:v>1.936</x:v>
+        <x:v>1.955</x:v>
       </x:c>
       <x:c r="H72" s="175" t="str">
         <x:v>logs/PBL6_R3_TRIP10_Manifest.postman_collection.log</x:v>
@@ -6795,7 +6795,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G73" s="173" t="n">
-        <x:v>2.027</x:v>
+        <x:v>1.849</x:v>
       </x:c>
       <x:c r="H73" s="175" t="str">
         <x:v>logs/PBL6_R3_TRIP12_CancelSoldTrip.postman_collection.log</x:v>
@@ -6824,7 +6824,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G74" s="173" t="n">
-        <x:v>1.938</x:v>
+        <x:v>2.077</x:v>
       </x:c>
       <x:c r="H74" s="175" t="str">
         <x:v>logs/PBL6_R3_TRIP12_SoldTripReadback.postman_collection.log</x:v>
@@ -6853,7 +6853,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G75" s="173" t="n">
-        <x:v>2.101</x:v>
+        <x:v>2.024</x:v>
       </x:c>
       <x:c r="H75" s="175" t="str">
         <x:v>logs/PBL6_R3_TripCancel.postman_collection.log</x:v>
@@ -6882,7 +6882,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G76" s="173" t="n">
-        <x:v>1.822</x:v>
+        <x:v>1.923</x:v>
       </x:c>
       <x:c r="H76" s="175" t="str">
         <x:v>logs/PBL6_R3_TripReadback.postman_collection.log</x:v>
@@ -6911,7 +6911,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G77" s="173" t="n">
-        <x:v>2.071</x:v>
+        <x:v>2.139</x:v>
       </x:c>
       <x:c r="H77" s="175" t="str">
         <x:v>logs/PBL6_R3_Trips.postman_collection.log</x:v>
@@ -6940,7 +6940,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G78" s="173" t="n">
-        <x:v>2.401</x:v>
+        <x:v>2.66</x:v>
       </x:c>
       <x:c r="H78" s="175" t="str">
         <x:v>logs/PBL6_R3_TripState.postman_collection.log</x:v>
@@ -6969,7 +6969,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G79" s="173" t="n">
-        <x:v>1.799</x:v>
+        <x:v>2.301</x:v>
       </x:c>
       <x:c r="H79" s="175" t="str">
         <x:v>logs/PBL6_R3_UnknownTicket.postman_collection.log</x:v>
@@ -6998,7 +6998,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G80" s="173" t="n">
-        <x:v>1.803</x:v>
+        <x:v>2.006</x:v>
       </x:c>
       <x:c r="H80" s="175" t="str">
         <x:v>logs/PBL6_REP02_ReadOnly_Smoke.postman_collection.log</x:v>
@@ -7018,16 +7018,16 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="D81" s="173" t="n">
-        <x:v>66</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E81" s="173" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F81" s="173" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G81" s="173" t="n">
-        <x:v>3.223</x:v>
+        <x:v>3.181</x:v>
       </x:c>
       <x:c r="H81" s="175" t="str">
         <x:v>logs/PBL6_SEC01_Protected_Endpoint_Matrix.postman_collection.log</x:v>
@@ -7056,7 +7056,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G82" s="173" t="n">
-        <x:v>7.582</x:v>
+        <x:v>7.778</x:v>
       </x:c>
       <x:c r="H82" s="175" t="str">
         <x:v>logs/PBL6_Workbook_API_Verification.postman_collection.log</x:v>
@@ -7925,10 +7925,10 @@
         <x:v>Auth Service</x:v>
       </x:c>
       <x:c r="D11" s="69" t="n">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="E11" s="69" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F11" s="69" t="n">
         <x:v>2</x:v>
@@ -8064,10 +8064,10 @@
         <x:v>Sub total</x:v>
       </x:c>
       <x:c r="D18" s="73" t="n">
-        <x:v>95</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E18" s="73" t="n">
-        <x:v>31</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F18" s="73" t="n">
         <x:v>11</x:v>
@@ -8098,7 +8098,7 @@
       </x:c>
       <x:c r="E21" s="158" t="n">
         <x:f>D18/H18</x:f>
-        <x:v>0.6209150326797386</x:v>
+        <x:v>0.6274509803921569</x:v>
       </x:c>
       <x:c r="F21" s="7" t="s">
         <x:v>106</x:v>
@@ -8328,10 +8328,10 @@
         <x:v>Auth Service</x:v>
       </x:c>
       <x:c r="D36" s="69" t="n">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="E36" s="69" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F36" s="69" t="n">
         <x:v>2</x:v>
@@ -8464,10 +8464,10 @@
         <x:v>Sub total</x:v>
       </x:c>
       <x:c r="D42" s="73" t="n">
-        <x:v>95</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E42" s="73" t="n">
-        <x:v>31</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F42" s="73" t="n">
         <x:v>11</x:v>
@@ -8744,10 +8744,10 @@
         <x:v>Round 2</x:v>
       </x:c>
       <x:c r="B7" s="90" t="n">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C7" s="90" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D7" s="90" t="n">
         <x:v>2</x:v>
@@ -10354,7 +10354,7 @@
         <x:v>Minh Trí</x:v>
       </x:c>
       <x:c r="I51" s="152" t="str">
-        <x:v>Failed</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J51" s="145" t="n">
         <x:v>46325</x:v>
@@ -10366,7 +10366,7 @@
       <x:c r="M51" s="145"/>
       <x:c r="N51" s="101"/>
       <x:c r="O51" s="155" t="str">
-        <x:v>Round 2: chưa đạt; xem collection log tương ứng trong outputs/pbl6-round2/logs.</x:v>
+        <x:v>Round 2: đạt; có bằng chứng trong Postman log/JUnit.</x:v>
       </x:c>
       <x:c r="Q51" s="100"/>
     </x:row>
@@ -11069,7 +11069,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ae780ba1d4d4afe"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba018c7daddf42b9"/>
 </x:worksheet>
 </file>
 
@@ -13559,7 +13559,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb60c01af4244d35"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9733c2509da2440d"/>
 </x:worksheet>
 </file>
 
@@ -16467,7 +16467,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1be63b6599ba4367"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fab1f8cf1734c93"/>
 </x:worksheet>
 </file>
 
@@ -18167,7 +18167,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72061d571b364091"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c2ca3b75bc14e3d"/>
 </x:worksheet>
 </file>
 
@@ -19535,7 +19535,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R755ae62f14e940c2"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fff5364bb8143e0"/>
 </x:worksheet>
 </file>
 
@@ -21025,6 +21025,6 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R239e2e7168254373"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22abdc13317e4f2b"/>
 </x:worksheet>
 </file>
</xml_diff>